<commit_message>
added test and evaluations
</commit_message>
<xml_diff>
--- a/memo_evaluation_results/cost.xlsx
+++ b/memo_evaluation_results/cost.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ak/Desktop/Final/Submission_VC_Agents/memo_evaluation_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EBB4CF3-38FF-D840-85D3-D100BF1DAB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{982EA95D-2361-D94A-98A8-AEC652DCCDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15840" xr2:uid="{93B05559-0107-6D4A-830C-B103A6EDCF5F}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15700" xr2:uid="{93B05559-0107-6D4A-830C-B103A6EDCF5F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029" refMode="R1C1"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
   <si>
     <t>before run</t>
   </si>
@@ -231,6 +231,27 @@
   </si>
   <si>
     <t>$7.93</t>
+  </si>
+  <si>
+    <t>$10.58</t>
+  </si>
+  <si>
+    <t>$11.23</t>
+  </si>
+  <si>
+    <t>$4.17</t>
+  </si>
+  <si>
+    <t>before 40 runs</t>
+  </si>
+  <si>
+    <t>after</t>
+  </si>
+  <si>
+    <t>$3.71</t>
+  </si>
+  <si>
+    <t>$7.48</t>
   </si>
 </sst>
 </file>
@@ -238,9 +259,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="[$USD]\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$USD]\ #,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -254,13 +275,6 @@
       <name val="RedHatText"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -293,10 +307,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1129,6 +1143,294 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 1" descr="download">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02BEF9CE-AE79-6779-C08C-7AAB2E060A0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="20904200" y="2489200"/>
+          <a:ext cx="254000" cy="254000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="AutoShape 2" descr="search">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA5445D5-B38D-EDDB-6AC3-D121DD3568EF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="20904200" y="2946400"/>
+          <a:ext cx="254000" cy="254000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 3" descr="download">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8DE828B-20BC-65BE-9A44-C4D235AD608B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="20904200" y="2489200"/>
+          <a:ext cx="254000" cy="254000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="AutoShape 4" descr="search">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E7BEA94-5909-8796-4F27-6CD8B5A4F455}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="20904200" y="2946400"/>
+          <a:ext cx="254000" cy="254000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1029" name="AutoShape 5" descr="download">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D07E5C1D-19EE-086C-DC4A-29F53F9345E1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="22186900" y="2489200"/>
+          <a:ext cx="254000" cy="254000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1030" name="AutoShape 6" descr="search">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBF8A25A-3C6C-7761-98D1-BA790252FE78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="22186900" y="2946400"/>
+          <a:ext cx="254000" cy="254000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1449,7 +1751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DE69D48-A9B3-F34B-9111-E0A0683A0692}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="23.83203125" bestFit="1" customWidth="1"/>
@@ -1457,9 +1759,12 @@
     <col min="4" max="5" width="25.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="11" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:14">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1494,46 +1799,58 @@
       <c r="L1" s="2">
         <v>10</v>
       </c>
+      <c r="M1" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:14">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="M2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>67</v>
+      </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:14">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -1570,8 +1887,10 @@
       <c r="L3" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:14">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -1608,12 +1927,14 @@
       <c r="L4" s="2" t="s">
         <v>62</v>
       </c>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1646,8 +1967,14 @@
       <c r="L5" s="2" t="s">
         <v>63</v>
       </c>
+      <c r="M5" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:14">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -1684,9 +2011,11 @@
       <c r="L6" s="2">
         <v>546</v>
       </c>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:14">
+      <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1722,8 +2051,14 @@
       <c r="L7" s="2" t="s">
         <v>64</v>
       </c>
+      <c r="M7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>71</v>
+      </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:14">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
@@ -1760,9 +2095,11 @@
       <c r="L8" s="2">
         <v>85</v>
       </c>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:14">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="2"/>
@@ -1776,8 +2113,10 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:14">
       <c r="A10" s="2" t="s">
         <v>14</v>
       </c>
@@ -1814,8 +2153,14 @@
       <c r="L10" s="2">
         <v>494</v>
       </c>
+      <c r="M10" s="2">
+        <v>460</v>
+      </c>
+      <c r="N10" s="2">
+        <v>427</v>
+      </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:14">
       <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
@@ -1852,14 +2197,22 @@
       <c r="L11" s="2">
         <v>184</v>
       </c>
+      <c r="M11" s="2">
+        <v>147</v>
+      </c>
+      <c r="N11" s="2">
+        <v>117</v>
+      </c>
     </row>
-    <row r="12" spans="1:12" ht="18">
+    <row r="12" spans="1:14" ht="18">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>